<commit_message>
feat: Include 4 additional dashboard sheets into the global Native Excel Export
</commit_message>
<xml_diff>
--- a/public/templates/dashboard_template_all.xlsx
+++ b/public/templates/dashboard_template_all.xlsx
@@ -9,15 +9,19 @@
   <sheets>
     <sheet name="Dashboard Profil" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard PRB" sheetId="2" r:id="rId2"/>
-    <sheet name="Dashboard Home Care" sheetId="3" r:id="rId3"/>
-    <sheet name="Dashboard Paliatif" sheetId="4" r:id="rId4"/>
+    <sheet name="Dashboard Monitoring PRB" sheetId="3" r:id="rId3"/>
+    <sheet name="Dashboard Home Care" sheetId="4" r:id="rId4"/>
+    <sheet name="Dashboard Paliatif" sheetId="5" r:id="rId5"/>
+    <sheet name="Dashboard Non-Optimal" sheetId="6" r:id="rId6"/>
+    <sheet name="Dashboard Sp.KKLP" sheetId="7" r:id="rId7"/>
+    <sheet name="Dashboard Kendala" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="77">
   <si>
     <t>DASHBOARD PROFIL RESPONDEN</t>
   </si>
@@ -193,15 +197,21 @@
     <t>Penyakit 9</t>
   </si>
   <si>
+    <t>DASHBOARD MONITORING PRB</t>
+  </si>
+  <si>
+    <t>FKTP dengan Mekanisme (%)</t>
+  </si>
+  <si>
+    <t>Mekanisme</t>
+  </si>
+  <si>
     <t>DASHBOARD HOME CARE</t>
   </si>
   <si>
     <t>Proporsi FKTP dgn Home Care (%)</t>
   </si>
   <si>
-    <t>Rata-rata Kunjungan per Bulan</t>
-  </si>
-  <si>
     <t>Kondisi Pasien</t>
   </si>
   <si>
@@ -212,6 +222,36 @@
   </si>
   <si>
     <t>Tujuan Layanan</t>
+  </si>
+  <si>
+    <t>DASHBOARD NON-OPTIMAL</t>
+  </si>
+  <si>
+    <t>Total Identifikasi Non-Optimal</t>
+  </si>
+  <si>
+    <t>Status JKN</t>
+  </si>
+  <si>
+    <t>DASHBOARD PERAN SP.KKLP</t>
+  </si>
+  <si>
+    <t>Punya Dokter Sp.KKLP</t>
+  </si>
+  <si>
+    <t>Layanan Dirujuk</t>
+  </si>
+  <si>
+    <t>Diagnosis Sp.KKLP</t>
+  </si>
+  <si>
+    <t>DASHBOARD KENDALA JKN</t>
+  </si>
+  <si>
+    <t>FKTP dgn Kendala</t>
+  </si>
+  <si>
+    <t>Kendala</t>
   </si>
 </sst>
 </file>
@@ -385,6 +425,408 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Proporsi Masuk JKN</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard Non-Optimal'!$A$9:$A$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard Non-Optimal'!$B$9:$B$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Top 5 Layanan Dirujuk</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard Sp.KKLP'!$A$9:$A$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard Sp.KKLP'!$B$9:$B$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Diagnosis Sp.KKLP</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard Sp.KKLP'!$A$27:$A$36</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard Sp.KKLP'!$B$27:$B$36</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50120001"/>
+        <c:axId val="50120002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50120001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50120002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50120002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50120001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Distribusi Kendala</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard Kendala'!$A$9:$A$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard Kendala'!$B$9:$B$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50130001"/>
+        <c:axId val="50130002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50130001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50130002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50130002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50130001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
@@ -1044,7 +1486,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Kondisi Pasien Home Care</a:t>
+              <a:t>Mekanisme Utama PRB</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1060,19 +1502,19 @@
           <c:order val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'Dashboard Home Care'!$A$10:$A$15</c:f>
+              <c:f>'Dashboard Monitoring PRB'!$A$9:$A$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="5"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard Home Care'!$B$10:$B$15</c:f>
+              <c:f>'Dashboard Monitoring PRB'!$B$9:$B$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1086,9 +1528,6 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1123,6 +1562,99 @@
 </file>
 
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Kondisi Pasien Home Care</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard Home Care'!$A$10:$A$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard Home Care'!$B$10:$B$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
@@ -1411,6 +1943,41 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -1440,7 +2007,142 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2303,7 +3005,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -2347,20 +3049,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="2" t="s">
+    <row r="8" spans="1:12">
+      <c r="A8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B5">
-        <v>0</v>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>6</v>
+      <c r="B9">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2380,16 +3079,6 @@
     </row>
     <row r="13" spans="1:12">
       <c r="B13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="B14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
-      <c r="B15">
         <v>0</v>
       </c>
     </row>
@@ -2404,7 +3093,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -2412,7 +3101,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2442,7 +3131,100 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="2" t="s">
         <v>63</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="B15">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="30.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2450,7 +3232,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
@@ -2483,6 +3265,323 @@
     </row>
     <row r="14" spans="1:12">
       <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="30.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L36"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="30.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="B27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="B28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="B30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="B31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="B32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="30.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="B15">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add the remaining 5 tabs to the global excel download (Kualitatif, Keluhan, DPM, Pasien Bulanan, Raw Data)
</commit_message>
<xml_diff>
--- a/public/templates/dashboard_template_all.xlsx
+++ b/public/templates/dashboard_template_all.xlsx
@@ -15,13 +15,18 @@
     <sheet name="Dashboard Non-Optimal" sheetId="6" r:id="rId6"/>
     <sheet name="Dashboard Sp.KKLP" sheetId="7" r:id="rId7"/>
     <sheet name="Dashboard Kendala" sheetId="8" r:id="rId8"/>
+    <sheet name="Kualitatif" sheetId="9" r:id="rId9"/>
+    <sheet name="Keluhan" sheetId="10" r:id="rId10"/>
+    <sheet name="Dashboard DPM" sheetId="11" r:id="rId11"/>
+    <sheet name="Pasien Bulanan" sheetId="12" r:id="rId12"/>
+    <sheet name="Raw Data" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
   <si>
     <t>DASHBOARD PROFIL RESPONDEN</t>
   </si>
@@ -44,214 +49,142 @@
     <t>Jumlah</t>
   </si>
   <si>
-    <t>Puskesmas</t>
-  </si>
-  <si>
-    <t>Klinik</t>
-  </si>
-  <si>
-    <t>Dokter Praktik Mandiri</t>
-  </si>
-  <si>
-    <t>Unik</t>
+    <t>Tipe FKTP Unik</t>
   </si>
   <si>
     <t>Jabatan</t>
   </si>
   <si>
-    <t>Jabatan 0</t>
-  </si>
-  <si>
-    <t>Jabatan 1</t>
-  </si>
-  <si>
-    <t>Jabatan 2</t>
-  </si>
-  <si>
-    <t>Jabatan 3</t>
-  </si>
-  <si>
-    <t>Jabatan 4</t>
-  </si>
-  <si>
-    <t>Jabatan 5</t>
-  </si>
-  <si>
-    <t>Jabatan 6</t>
-  </si>
-  <si>
-    <t>Jabatan 7</t>
-  </si>
-  <si>
-    <t>Jabatan 8</t>
-  </si>
-  <si>
-    <t>Jabatan 9</t>
-  </si>
-  <si>
-    <t>Jabatan 10</t>
-  </si>
-  <si>
-    <t>Jabatan 11</t>
-  </si>
-  <si>
-    <t>Jabatan 12</t>
-  </si>
-  <si>
-    <t>Jabatan 13</t>
-  </si>
-  <si>
-    <t>Jabatan 14</t>
-  </si>
-  <si>
     <t>Provinsi</t>
   </si>
   <si>
-    <t>Provinsi 0</t>
-  </si>
-  <si>
-    <t>Provinsi 1</t>
-  </si>
-  <si>
-    <t>Provinsi 2</t>
-  </si>
-  <si>
-    <t>Provinsi 3</t>
-  </si>
-  <si>
-    <t>Provinsi 4</t>
-  </si>
-  <si>
-    <t>Provinsi 5</t>
-  </si>
-  <si>
-    <t>Provinsi 6</t>
-  </si>
-  <si>
-    <t>Provinsi 7</t>
-  </si>
-  <si>
-    <t>Provinsi 8</t>
-  </si>
-  <si>
-    <t>Provinsi 9</t>
-  </si>
-  <si>
-    <t>DASHBOARD PROGRAM RUJUK BALIK (PRB)</t>
-  </si>
-  <si>
-    <t>Total Estimasi Pasien PRB</t>
-  </si>
-  <si>
-    <t>Pasien PRB Rutin (Patuh)</t>
-  </si>
-  <si>
-    <t>Pasien PRB Tidak Berkunjung</t>
+    <t>DASHBOARD PRB</t>
+  </si>
+  <si>
+    <t>Total Pasien PRB</t>
+  </si>
+  <si>
+    <t>Rutin</t>
+  </si>
+  <si>
+    <t>Tidak Berkunjung</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Persentase (%)</t>
-  </si>
-  <si>
-    <t>Patuh Kunjungan</t>
-  </si>
-  <si>
-    <t>Tidak Patuh</t>
+    <t>Persentase</t>
   </si>
   <si>
     <t>Diagnosis</t>
   </si>
   <si>
-    <t>Jumlah FKTP</t>
-  </si>
-  <si>
-    <t>Penyakit 0</t>
-  </si>
-  <si>
-    <t>Penyakit 1</t>
-  </si>
-  <si>
-    <t>Penyakit 2</t>
-  </si>
-  <si>
-    <t>Penyakit 3</t>
-  </si>
-  <si>
-    <t>Penyakit 4</t>
-  </si>
-  <si>
-    <t>Penyakit 5</t>
-  </si>
-  <si>
-    <t>Penyakit 6</t>
-  </si>
-  <si>
-    <t>Penyakit 7</t>
-  </si>
-  <si>
-    <t>Penyakit 8</t>
-  </si>
-  <si>
-    <t>Penyakit 9</t>
-  </si>
-  <si>
-    <t>DASHBOARD MONITORING PRB</t>
-  </si>
-  <si>
-    <t>FKTP dengan Mekanisme (%)</t>
+    <t>MONITORING PRB</t>
+  </si>
+  <si>
+    <t>Mekanisme PRB (%)</t>
   </si>
   <si>
     <t>Mekanisme</t>
   </si>
   <si>
-    <t>DASHBOARD HOME CARE</t>
-  </si>
-  <si>
-    <t>Proporsi FKTP dgn Home Care (%)</t>
-  </si>
-  <si>
-    <t>Kondisi Pasien</t>
-  </si>
-  <si>
-    <t>DASHBOARD PALIATIF</t>
-  </si>
-  <si>
-    <t>Proporsi FKTP dgn Layanan Paliatif (%)</t>
-  </si>
-  <si>
-    <t>Tujuan Layanan</t>
-  </si>
-  <si>
-    <t>DASHBOARD NON-OPTIMAL</t>
-  </si>
-  <si>
-    <t>Total Identifikasi Non-Optimal</t>
-  </si>
-  <si>
-    <t>Status JKN</t>
-  </si>
-  <si>
-    <t>DASHBOARD PERAN SP.KKLP</t>
-  </si>
-  <si>
-    <t>Punya Dokter Sp.KKLP</t>
-  </si>
-  <si>
-    <t>Layanan Dirujuk</t>
-  </si>
-  <si>
-    <t>Diagnosis Sp.KKLP</t>
-  </si>
-  <si>
-    <t>DASHBOARD KENDALA JKN</t>
-  </si>
-  <si>
-    <t>FKTP dgn Kendala</t>
+    <t>HOME CARE</t>
+  </si>
+  <si>
+    <t>Proporsi HC (%)</t>
+  </si>
+  <si>
+    <t>Kondisi</t>
+  </si>
+  <si>
+    <t>PALIATIF</t>
+  </si>
+  <si>
+    <t>Proporsi Paliatif (%)</t>
+  </si>
+  <si>
+    <t>Tujuan</t>
+  </si>
+  <si>
+    <t>NON-OPTIMAL</t>
+  </si>
+  <si>
+    <t>Identifikasi</t>
+  </si>
+  <si>
+    <t>JKN</t>
+  </si>
+  <si>
+    <t>PERAN SP.KKLP</t>
+  </si>
+  <si>
+    <t>Punya SpKKLP</t>
+  </si>
+  <si>
+    <t>Rujukan</t>
+  </si>
+  <si>
+    <t>KENDALA JKN</t>
+  </si>
+  <si>
+    <t>Total Kendala</t>
   </si>
   <si>
     <t>Kendala</t>
+  </si>
+  <si>
+    <t>Nama Responden</t>
+  </si>
+  <si>
+    <t>Faskes</t>
+  </si>
+  <si>
+    <t>W1</t>
+  </si>
+  <si>
+    <t>W2</t>
+  </si>
+  <si>
+    <t>W3</t>
+  </si>
+  <si>
+    <t>W4</t>
+  </si>
+  <si>
+    <t>W5</t>
+  </si>
+  <si>
+    <t>W6</t>
+  </si>
+  <si>
+    <t>W7</t>
+  </si>
+  <si>
+    <t>W8</t>
+  </si>
+  <si>
+    <t>Keluhan</t>
+  </si>
+  <si>
+    <t>Solusi</t>
+  </si>
+  <si>
+    <t>DASHBOARD DPM</t>
+  </si>
+  <si>
+    <t>Lama Praktik</t>
+  </si>
+  <si>
+    <t>Kunjungan Harian</t>
+  </si>
+  <si>
+    <t>PASIEN BULANAN</t>
+  </si>
+  <si>
+    <t>Penyakit</t>
+  </si>
+  <si>
+    <t>Data will be populated by JS</t>
   </si>
 </sst>
 </file>
@@ -334,24 +267,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Proporsi Responden per FKTP</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -359,25 +274,14 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:dLbls>
-            <c:showPercent val="1"/>
-          </c:dLbls>
           <c:cat>
-            <c:strRef>
+            <c:numRef>
               <c:f>'Dashboard Profil'!$A$11:$A$13</c:f>
-              <c:strCache>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>Puskesmas</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Klinik</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Dokter Praktik Mandiri</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -429,24 +333,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Proporsi Masuk JKN</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -510,24 +396,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Top 5 Layanan Dirujuk</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -600,24 +468,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Diagnosis Sp.KKLP</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
@@ -706,6 +556,10 @@
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:printSettings>
@@ -720,24 +574,6 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Distribusi Kendala</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
@@ -817,6 +653,10 @@
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:printSettings>
@@ -827,28 +667,10 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Proporsi FKTP Unik</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -856,32 +678,21 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:dLbls>
-            <c:showPercent val="1"/>
-          </c:dLbls>
           <c:cat>
-            <c:strRef>
-              <c:f>'Dashboard Profil'!$A$27:$A$29</c:f>
-              <c:strCache>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>Puskesmas</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Klinik</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Dokter Praktik Mandiri</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:numRef>
+              <c:f>'Dashboard DPM'!$A$5:$A$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard Profil'!$B$27:$B$29</c:f>
+              <c:f>'Dashboard DPM'!$B$5:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -889,6 +700,12 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -922,28 +739,10 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Proporsi Jabatan</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -952,64 +751,20 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:strRef>
-              <c:f>'Dashboard Profil'!$A$43:$A$57</c:f>
-              <c:strCache>
-                <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>Jabatan 0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Jabatan 1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Jabatan 2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Jabatan 3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Jabatan 4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Jabatan 5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Jabatan 6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Jabatan 7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Jabatan 8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Jabatan 9</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Jabatan 10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Jabatan 11</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>Jabatan 12</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>Jabatan 13</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>Jabatan 14</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:numRef>
+              <c:f>'Dashboard DPM'!$A$27:$A$31</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard Profil'!$B$43:$B$57</c:f>
+              <c:f>'Dashboard DPM'!$B$27:$B$31</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1023,36 +778,6 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1086,80 +811,33 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>10 Provinsi Terbanyak</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="col"/>
+        <c:barDir val="bar"/>
         <c:grouping val="clustered"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:strRef>
-              <c:f>'Dashboard Profil'!$A$61:$A$70</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>Provinsi 0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Provinsi 1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Provinsi 2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Provinsi 3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Provinsi 4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Provinsi 5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Provinsi 6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Provinsi 7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Provinsi 8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Provinsi 9</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:numRef>
+              <c:f>'Pasien Bulanan'!$A$5:$A$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="16"/>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard Profil'!$B$61:$B$70</c:f>
+              <c:f>'Pasien Bulanan'!$B$5:$B$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1188,42 +866,65 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50040001"/>
-        <c:axId val="50040002"/>
+        <c:axId val="50160001"/>
+        <c:axId val="50160002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50040001"/>
+        <c:axId val="50160001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50040002"/>
+        <c:crossAx val="50160002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50040002"/>
+        <c:axId val="50160002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50040001"/>
+        <c:crossAx val="50160001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:printSettings>
@@ -1234,28 +935,10 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Kepatuhan Kunjungan PRB</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -1263,33 +946,28 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:dLbls>
-            <c:showPercent val="1"/>
-          </c:dLbls>
           <c:cat>
-            <c:strRef>
-              <c:f>'Dashboard PRB'!$A$11:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>Patuh Kunjungan</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Tidak Patuh</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:numRef>
+              <c:f>'Dashboard Profil'!$A$27:$A$29</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard PRB'!$B$11:$B$12</c:f>
+              <c:f>'Dashboard Profil'!$B$27:$B$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1323,176 +1001,10 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Diagnosis PRB Terbanyak</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="bar"/>
-        <c:grouping val="clustered"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Dashboard PRB'!$A$27:$A$36</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>Penyakit 0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Penyakit 1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Penyakit 2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Penyakit 3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Penyakit 4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Penyakit 5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Penyakit 6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Penyakit 7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Penyakit 8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Penyakit 9</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Dashboard PRB'!$B$27:$B$36</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:axId val="50060001"/>
-        <c:axId val="50060002"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="50060001"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:axPos val="l"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50060002"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="50060002"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:axPos val="b"/>
-        <c:majorGridlines/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50060001"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-  </c:chart>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:lang val="en-US"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Mekanisme Utama PRB</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:layout/>
-    </c:title>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -1502,19 +1014,19 @@
           <c:order val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'Dashboard Monitoring PRB'!$A$9:$A$13</c:f>
+              <c:f>'Dashboard Profil'!$A$43:$A$57</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="15"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard Monitoring PRB'!$B$9:$B$13</c:f>
+              <c:f>'Dashboard Profil'!$B$43:$B$57</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1528,6 +1040,36 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1561,28 +1103,116 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Kondisi Pasien Home Care</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
+    <c:plotArea>
       <c:layout/>
-    </c:title>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard Profil'!$A$61:$A$70</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard Profil'!$B$61:$B$70</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50040001"/>
+        <c:axId val="50040002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50040001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50040002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50040002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50040001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -1592,35 +1222,23 @@
           <c:order val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'Dashboard Home Care'!$A$10:$A$15</c:f>
+              <c:f>'Dashboard PRB'!$A$11:$A$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="2"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard Home Care'!$B$10:$B$15</c:f>
+              <c:f>'Dashboard PRB'!$B$11:$B$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1654,28 +1272,116 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Tujuan Layanan Paliatif</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
+    <c:plotArea>
       <c:layout/>
-    </c:title>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard PRB'!$A$27:$A$36</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard PRB'!$B$27:$B$36</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50060001"/>
+        <c:axId val="50060002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50060001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50060002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50060002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50060001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -1685,19 +1391,19 @@
           <c:order val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'Dashboard Paliatif'!$A$9:$A$14</c:f>
+              <c:f>'Dashboard Monitoring PRB'!$A$9:$A$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="5"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard Paliatif'!$B$9:$B$14</c:f>
+              <c:f>'Dashboard Monitoring PRB'!$B$9:$B$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1711,9 +1417,6 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1747,6 +1450,156 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard Home Care'!$A$10:$A$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard Home Care'!$B$10:$B$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Dashboard Paliatif'!$A$9:$A$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Dashboard Paliatif'!$B$9:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1757,8 +1610,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -1787,8 +1640,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -1817,8 +1670,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>55</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -1847,8 +1700,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>73</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -1864,6 +1717,41 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2169,6 +2057,71 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2465,8 +2418,7 @@
   <dimension ref="A1:L70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="25.7109375" customWidth="1"/>
-    <col min="4" max="11" width="15.7109375" customWidth="1"/>
+    <col min="1" max="2" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -2540,273 +2492,180 @@
       </c>
     </row>
     <row r="11" spans="1:12">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
       <c r="B13">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" t="s">
-        <v>7</v>
-      </c>
       <c r="B27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" t="s">
-        <v>8</v>
-      </c>
       <c r="B28">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" t="s">
-        <v>9</v>
-      </c>
       <c r="B29">
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" t="s">
-        <v>12</v>
-      </c>
       <c r="B43">
         <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" t="s">
-        <v>13</v>
-      </c>
       <c r="B44">
         <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" t="s">
-        <v>14</v>
-      </c>
       <c r="B45">
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" t="s">
-        <v>15</v>
-      </c>
       <c r="B46">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" t="s">
-        <v>16</v>
-      </c>
       <c r="B47">
         <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" t="s">
-        <v>17</v>
-      </c>
       <c r="B48">
         <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" t="s">
-        <v>18</v>
-      </c>
       <c r="B49">
         <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:2">
-      <c r="A50" t="s">
-        <v>19</v>
-      </c>
       <c r="B50">
         <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:2">
-      <c r="A51" t="s">
-        <v>20</v>
-      </c>
       <c r="B51">
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:2">
-      <c r="A52" t="s">
-        <v>21</v>
-      </c>
       <c r="B52">
         <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:2">
-      <c r="A53" t="s">
-        <v>22</v>
-      </c>
       <c r="B53">
         <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:2">
-      <c r="A54" t="s">
-        <v>23</v>
-      </c>
       <c r="B54">
         <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:2">
-      <c r="A55" t="s">
-        <v>24</v>
-      </c>
       <c r="B55">
         <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:2">
-      <c r="A56" t="s">
-        <v>25</v>
-      </c>
       <c r="B56">
         <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:2">
-      <c r="A57" t="s">
-        <v>26</v>
-      </c>
       <c r="B57">
         <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:2">
-      <c r="A61" t="s">
-        <v>28</v>
-      </c>
       <c r="B61">
         <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:2">
-      <c r="A62" t="s">
-        <v>29</v>
-      </c>
       <c r="B62">
         <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:2">
-      <c r="A63" t="s">
-        <v>30</v>
-      </c>
       <c r="B63">
         <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:2">
-      <c r="A64" t="s">
-        <v>31</v>
-      </c>
       <c r="B64">
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
-      <c r="A65" t="s">
-        <v>32</v>
-      </c>
+    <row r="65" spans="2:2">
       <c r="B65">
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
-      <c r="A66" t="s">
-        <v>33</v>
-      </c>
+    <row r="66" spans="2:2">
       <c r="B66">
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
-      <c r="A67" t="s">
-        <v>34</v>
-      </c>
+    <row r="67" spans="2:2">
       <c r="B67">
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
-      <c r="A68" t="s">
-        <v>35</v>
-      </c>
+    <row r="68" spans="2:2">
       <c r="B68">
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
-      <c r="A69" t="s">
-        <v>36</v>
-      </c>
+    <row r="69" spans="2:2">
       <c r="B69">
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
-      <c r="A70" t="s">
-        <v>37</v>
-      </c>
+    <row r="70" spans="2:2">
       <c r="B70">
         <v>0</v>
       </c>
@@ -2820,17 +2679,44 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="25.7109375" customWidth="1"/>
+    <col min="3" max="4" width="60.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2860,137 +2746,67 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
+        <v>48</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:12">
-      <c r="A5" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="B5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="B6">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
-      <c r="A10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="A11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12">
+    <row r="7" spans="1:12">
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="B9">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>47</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" t="s">
-        <v>48</v>
-      </c>
       <c r="B27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" t="s">
-        <v>49</v>
-      </c>
       <c r="B28">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" t="s">
-        <v>50</v>
-      </c>
       <c r="B29">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" t="s">
-        <v>51</v>
-      </c>
       <c r="B30">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" t="s">
-        <v>52</v>
-      </c>
       <c r="B31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="A32" t="s">
-        <v>53</v>
-      </c>
-      <c r="B32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2">
-      <c r="A33" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2">
-      <c r="A34" t="s">
-        <v>55</v>
-      </c>
-      <c r="B34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2">
-      <c r="A35" t="s">
-        <v>56</v>
-      </c>
-      <c r="B35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
-      <c r="A36" t="s">
-        <v>57</v>
-      </c>
-      <c r="B36">
         <v>0</v>
       </c>
     </row>
@@ -3003,9 +2819,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -3013,7 +2829,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3043,18 +2859,30 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4">
+        <v>51</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="B7">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>6</v>
+      <c r="B8">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -3079,6 +2907,41 @@
     </row>
     <row r="13" spans="1:12">
       <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="B15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="B16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20">
         <v>0</v>
       </c>
     </row>
@@ -3091,9 +2954,24 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -3101,7 +2979,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3131,23 +3009,34 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>6</v>
+    <row r="5" spans="1:12">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
-      <c r="B10">
-        <v>0</v>
+      <c r="A10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -3160,18 +3049,61 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
-      <c r="B13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="B14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
-      <c r="B15">
+    <row r="26" spans="1:2">
+      <c r="A26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="B27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="B28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="B30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="B31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="B32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36">
         <v>0</v>
       </c>
     </row>
@@ -3184,9 +3116,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -3194,7 +3126,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3224,7 +3156,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3232,7 +3164,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
@@ -3260,11 +3192,6 @@
     </row>
     <row r="13" spans="1:12">
       <c r="B13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="B14">
         <v>0</v>
       </c>
     </row>
@@ -3277,9 +3204,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -3287,7 +3214,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3317,27 +3244,47 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
-      <c r="A8" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="2" t="s">
+    <row r="9" spans="1:12">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="B9">
-        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="B15">
         <v>0</v>
       </c>
     </row>
@@ -3350,9 +3297,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -3360,7 +3307,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3390,7 +3337,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3398,7 +3345,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
@@ -3429,61 +3376,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
-      <c r="A26" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="B27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
-      <c r="B28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
-      <c r="B29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
-      <c r="B30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2">
-      <c r="B31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="B32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="2:2">
-      <c r="B33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2">
-      <c r="B34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2">
-      <c r="B35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="2:2">
-      <c r="B36">
+    <row r="14" spans="1:12">
+      <c r="B14">
         <v>0</v>
       </c>
     </row>
@@ -3496,9 +3390,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -3506,7 +3400,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3536,7 +3430,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>75</v>
+        <v>27</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3544,7 +3438,7 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
@@ -3557,31 +3451,6 @@
     </row>
     <row r="10" spans="1:12">
       <c r="B10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="B11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="B12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="B13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="B14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
-      <c r="B15">
         <v>0</v>
       </c>
     </row>
@@ -3592,4 +3461,293 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L36"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="30.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="B27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="B28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="B30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="B31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="B32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="30.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="B15">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="10" width="50.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: Rewrite python excel template generators with placeholder strings to prevent chart corruption in xlsx-populate and fix template cache busting
</commit_message>
<xml_diff>
--- a/public/templates/dashboard_template_all.xlsx
+++ b/public/templates/dashboard_template_all.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="139">
   <si>
     <t>DASHBOARD PROFIL RESPONDEN</t>
   </si>
@@ -49,15 +49,99 @@
     <t>Jumlah</t>
   </si>
   <si>
+    <t>Puskesmas</t>
+  </si>
+  <si>
+    <t>Klinik</t>
+  </si>
+  <si>
+    <t>Dokter Praktik Mandiri</t>
+  </si>
+  <si>
     <t>Tipe FKTP Unik</t>
   </si>
   <si>
     <t>Jabatan</t>
   </si>
   <si>
+    <t>Jabatan 1</t>
+  </si>
+  <si>
+    <t>Jabatan 2</t>
+  </si>
+  <si>
+    <t>Jabatan 3</t>
+  </si>
+  <si>
+    <t>Jabatan 4</t>
+  </si>
+  <si>
+    <t>Jabatan 5</t>
+  </si>
+  <si>
+    <t>Jabatan 6</t>
+  </si>
+  <si>
+    <t>Jabatan 7</t>
+  </si>
+  <si>
+    <t>Jabatan 8</t>
+  </si>
+  <si>
+    <t>Jabatan 9</t>
+  </si>
+  <si>
+    <t>Jabatan 10</t>
+  </si>
+  <si>
+    <t>Jabatan 11</t>
+  </si>
+  <si>
+    <t>Jabatan 12</t>
+  </si>
+  <si>
+    <t>Jabatan 13</t>
+  </si>
+  <si>
+    <t>Jabatan 14</t>
+  </si>
+  <si>
+    <t>Jabatan 15</t>
+  </si>
+  <si>
     <t>Provinsi</t>
   </si>
   <si>
+    <t>Provinsi 1</t>
+  </si>
+  <si>
+    <t>Provinsi 2</t>
+  </si>
+  <si>
+    <t>Provinsi 3</t>
+  </si>
+  <si>
+    <t>Provinsi 4</t>
+  </si>
+  <si>
+    <t>Provinsi 5</t>
+  </si>
+  <si>
+    <t>Provinsi 6</t>
+  </si>
+  <si>
+    <t>Provinsi 7</t>
+  </si>
+  <si>
+    <t>Provinsi 8</t>
+  </si>
+  <si>
+    <t>Provinsi 9</t>
+  </si>
+  <si>
+    <t>Provinsi 10</t>
+  </si>
+  <si>
     <t>DASHBOARD PRB</t>
   </si>
   <si>
@@ -79,6 +163,36 @@
     <t>Diagnosis</t>
   </si>
   <si>
+    <t>Penyakit 1</t>
+  </si>
+  <si>
+    <t>Penyakit 2</t>
+  </si>
+  <si>
+    <t>Penyakit 3</t>
+  </si>
+  <si>
+    <t>Penyakit 4</t>
+  </si>
+  <si>
+    <t>Penyakit 5</t>
+  </si>
+  <si>
+    <t>Penyakit 6</t>
+  </si>
+  <si>
+    <t>Penyakit 7</t>
+  </si>
+  <si>
+    <t>Penyakit 8</t>
+  </si>
+  <si>
+    <t>Penyakit 9</t>
+  </si>
+  <si>
+    <t>Penyakit 10</t>
+  </si>
+  <si>
     <t>MONITORING PRB</t>
   </si>
   <si>
@@ -88,6 +202,21 @@
     <t>Mekanisme</t>
   </si>
   <si>
+    <t>Mek 1</t>
+  </si>
+  <si>
+    <t>Mek 2</t>
+  </si>
+  <si>
+    <t>Mek 3</t>
+  </si>
+  <si>
+    <t>Mek 4</t>
+  </si>
+  <si>
+    <t>Mek 5</t>
+  </si>
+  <si>
     <t>HOME CARE</t>
   </si>
   <si>
@@ -97,6 +226,24 @@
     <t>Kondisi</t>
   </si>
   <si>
+    <t>Kondisi 1</t>
+  </si>
+  <si>
+    <t>Kondisi 2</t>
+  </si>
+  <si>
+    <t>Kondisi 3</t>
+  </si>
+  <si>
+    <t>Kondisi 4</t>
+  </si>
+  <si>
+    <t>Kondisi 5</t>
+  </si>
+  <si>
+    <t>Kondisi 6</t>
+  </si>
+  <si>
     <t>PALIATIF</t>
   </si>
   <si>
@@ -106,6 +253,24 @@
     <t>Tujuan</t>
   </si>
   <si>
+    <t>Tujuan 1</t>
+  </si>
+  <si>
+    <t>Tujuan 2</t>
+  </si>
+  <si>
+    <t>Tujuan 3</t>
+  </si>
+  <si>
+    <t>Tujuan 4</t>
+  </si>
+  <si>
+    <t>Tujuan 5</t>
+  </si>
+  <si>
+    <t>Tujuan 6</t>
+  </si>
+  <si>
     <t>NON-OPTIMAL</t>
   </si>
   <si>
@@ -115,6 +280,12 @@
     <t>JKN</t>
   </si>
   <si>
+    <t>Diusulkan Masuk JKN</t>
+  </si>
+  <si>
+    <t>Tidak Diusulkan</t>
+  </si>
+  <si>
     <t>PERAN SP.KKLP</t>
   </si>
   <si>
@@ -124,6 +295,21 @@
     <t>Rujukan</t>
   </si>
   <si>
+    <t>Rujukan 1</t>
+  </si>
+  <si>
+    <t>Rujukan 2</t>
+  </si>
+  <si>
+    <t>Rujukan 3</t>
+  </si>
+  <si>
+    <t>Rujukan 4</t>
+  </si>
+  <si>
+    <t>Rujukan 5</t>
+  </si>
+  <si>
     <t>KENDALA JKN</t>
   </si>
   <si>
@@ -133,6 +319,27 @@
     <t>Kendala</t>
   </si>
   <si>
+    <t>Kendala 1</t>
+  </si>
+  <si>
+    <t>Kendala 2</t>
+  </si>
+  <si>
+    <t>Kendala 3</t>
+  </si>
+  <si>
+    <t>Kendala 4</t>
+  </si>
+  <si>
+    <t>Kendala 5</t>
+  </si>
+  <si>
+    <t>Kendala 6</t>
+  </si>
+  <si>
+    <t>Kendala 7</t>
+  </si>
+  <si>
     <t>Nama Responden</t>
   </si>
   <si>
@@ -175,16 +382,67 @@
     <t>Lama Praktik</t>
   </si>
   <si>
+    <t>Durasi 1</t>
+  </si>
+  <si>
+    <t>Durasi 2</t>
+  </si>
+  <si>
+    <t>Durasi 3</t>
+  </si>
+  <si>
+    <t>Durasi 4</t>
+  </si>
+  <si>
+    <t>Durasi 5</t>
+  </si>
+  <si>
     <t>Kunjungan Harian</t>
   </si>
   <si>
+    <t>Range 1</t>
+  </si>
+  <si>
+    <t>Range 2</t>
+  </si>
+  <si>
+    <t>Range 3</t>
+  </si>
+  <si>
+    <t>Range 4</t>
+  </si>
+  <si>
+    <t>Range 5</t>
+  </si>
+  <si>
     <t>PASIEN BULANAN</t>
   </si>
   <si>
     <t>Penyakit</t>
   </si>
   <si>
-    <t>Data will be populated by JS</t>
+    <t>Penyakit 11</t>
+  </si>
+  <si>
+    <t>Penyakit 12</t>
+  </si>
+  <si>
+    <t>Penyakit 13</t>
+  </si>
+  <si>
+    <t>Penyakit 14</t>
+  </si>
+  <si>
+    <t>Penyakit 15</t>
+  </si>
+  <si>
+    <t>Penyakit 16</t>
+  </si>
+  <si>
+    <t>Waktu Submit</t>
+  </si>
+  <si>
+    <t>Kab/Kota</t>
   </si>
 </sst>
 </file>
@@ -275,13 +533,21 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Profil'!$A$11:$A$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="3"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Puskesmas</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Klinik</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Dokter Praktik Mandiri</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -341,13 +607,18 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Non-Optimal'!$A$9:$A$10</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Diusulkan Masuk JKN</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Tidak Diusulkan</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -404,13 +675,27 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Sp.KKLP'!$A$9:$A$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="5"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Rujukan 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Rujukan 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Rujukan 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Rujukan 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Rujukan 5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -477,13 +762,42 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Sp.KKLP'!$A$27:$A$36</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="10"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Penyakit 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Penyakit 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Penyakit 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Penyakit 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Penyakit 5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Penyakit 6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Penyakit 7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Penyakit 8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Penyakit 9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Penyakit 10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -534,7 +848,6 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50120002"/>
         <c:crosses val="autoZero"/>
@@ -583,13 +896,33 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Kendala'!$A$9:$A$15</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="7"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Kendala 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Kendala 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Kendala 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Kendala 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Kendala 5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Kendala 6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Kendala 7</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -631,7 +964,6 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50130002"/>
         <c:crosses val="autoZero"/>
@@ -679,13 +1011,27 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard DPM'!$A$5:$A$9</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="5"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Durasi 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Durasi 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Durasi 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Durasi 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Durasi 5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -751,13 +1097,27 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard DPM'!$A$27:$A$31</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="5"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Range 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Range 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Range 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Range 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Range 5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -824,13 +1184,60 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Pasien Bulanan'!$A$5:$A$20</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="16"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Penyakit 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Penyakit 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Penyakit 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Penyakit 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Penyakit 5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Penyakit 6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Penyakit 7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Penyakit 8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Penyakit 9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Penyakit 10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Penyakit 11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Penyakit 12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Penyakit 13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Penyakit 14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Penyakit 15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Penyakit 16</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -899,7 +1306,6 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50160002"/>
         <c:crosses val="autoZero"/>
@@ -947,13 +1353,21 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Profil'!$A$27:$A$29</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="3"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Puskesmas</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Klinik</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Dokter Praktik Mandiri</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1013,13 +1427,57 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Profil'!$A$43:$A$57</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="15"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Jabatan 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Jabatan 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Jabatan 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Jabatan 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Jabatan 5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jabatan 6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jabatan 7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Jabatan 8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Jabatan 9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Jabatan 10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Jabatan 11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Jabatan 12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jabatan 13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Jabatan 14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Jabatan 15</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1116,13 +1574,42 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Profil'!$A$61:$A$70</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="10"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Provinsi 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Provinsi 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Provinsi 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Provinsi 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Provinsi 5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Provinsi 6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Provinsi 7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Provinsi 8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Provinsi 9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Provinsi 10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1173,7 +1660,6 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50040002"/>
         <c:crosses val="autoZero"/>
@@ -1221,13 +1707,18 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard PRB'!$A$11:$A$12</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="2"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Rutin</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Tidak Berkunjung</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1285,13 +1776,42 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard PRB'!$A$27:$A$36</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="10"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Penyakit 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Penyakit 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Penyakit 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Penyakit 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Penyakit 5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Penyakit 6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Penyakit 7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Penyakit 8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Penyakit 9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Penyakit 10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1342,7 +1862,6 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50060002"/>
         <c:crosses val="autoZero"/>
@@ -1390,13 +1909,27 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Monitoring PRB'!$A$9:$A$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="5"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Mek 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Mek 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mek 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mek 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Mek 5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1462,13 +1995,30 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Home Care'!$A$10:$A$15</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="6"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Kondisi 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Kondisi 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Kondisi 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Kondisi 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Kondisi 5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Kondisi 6</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1537,13 +2087,30 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:cat>
-            <c:numRef>
+            <c:strRef>
               <c:f>'Dashboard Paliatif'!$A$9:$A$14</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
+              <c:strCache>
                 <c:ptCount val="6"/>
-              </c:numCache>
-            </c:numRef>
+                <c:pt idx="0">
+                  <c:v>Tujuan 1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Tujuan 2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Tujuan 3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Tujuan 4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Tujuan 5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Tujuan 6</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -2492,180 +3059,273 @@
       </c>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
       <c r="B13">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
       <c r="B27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>8</v>
+      </c>
       <c r="B28">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>9</v>
+      </c>
       <c r="B29">
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:2">
+      <c r="A43" t="s">
+        <v>12</v>
+      </c>
       <c r="B43">
         <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>13</v>
+      </c>
       <c r="B44">
         <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>14</v>
+      </c>
       <c r="B45">
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>15</v>
+      </c>
       <c r="B46">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:2">
+      <c r="A47" t="s">
+        <v>16</v>
+      </c>
       <c r="B47">
         <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:2">
+      <c r="A48" t="s">
+        <v>17</v>
+      </c>
       <c r="B48">
         <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>18</v>
+      </c>
       <c r="B49">
         <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>19</v>
+      </c>
       <c r="B50">
         <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>20</v>
+      </c>
       <c r="B51">
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:2">
+      <c r="A52" t="s">
+        <v>21</v>
+      </c>
       <c r="B52">
         <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>22</v>
+      </c>
       <c r="B53">
         <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>23</v>
+      </c>
       <c r="B54">
         <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:2">
+      <c r="A55" t="s">
+        <v>24</v>
+      </c>
       <c r="B55">
         <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:2">
+      <c r="A56" t="s">
+        <v>25</v>
+      </c>
       <c r="B56">
         <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:2">
+      <c r="A57" t="s">
+        <v>26</v>
+      </c>
       <c r="B57">
         <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>28</v>
+      </c>
       <c r="B61">
         <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:2">
+      <c r="A62" t="s">
+        <v>29</v>
+      </c>
       <c r="B62">
         <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:2">
+      <c r="A63" t="s">
+        <v>30</v>
+      </c>
       <c r="B63">
         <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>31</v>
+      </c>
       <c r="B64">
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
+        <v>32</v>
+      </c>
       <c r="B65">
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="1:2">
+      <c r="A66" t="s">
+        <v>33</v>
+      </c>
       <c r="B66">
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="1:2">
+      <c r="A67" t="s">
+        <v>34</v>
+      </c>
       <c r="B67">
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
+        <v>35</v>
+      </c>
       <c r="B68">
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
+        <v>36</v>
+      </c>
       <c r="B69">
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
+        <v>37</v>
+      </c>
       <c r="B70">
         <v>0</v>
       </c>
@@ -2689,16 +3349,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>35</v>
+        <v>104</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>45</v>
+        <v>114</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>46</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2716,7 +3376,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>116</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2746,66 +3406,96 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>48</v>
+        <v>117</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>118</v>
+      </c>
       <c r="B5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>119</v>
+      </c>
       <c r="B6">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>120</v>
+      </c>
       <c r="B7">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>121</v>
+      </c>
       <c r="B8">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>122</v>
+      </c>
       <c r="B9">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
-        <v>49</v>
+        <v>123</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>124</v>
+      </c>
       <c r="B27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>125</v>
+      </c>
       <c r="B28">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>126</v>
+      </c>
       <c r="B29">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>127</v>
+      </c>
       <c r="B30">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>128</v>
+      </c>
       <c r="B31">
         <v>0</v>
       </c>
@@ -2829,7 +3519,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>129</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2859,88 +3549,136 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>51</v>
+        <v>130</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
       <c r="B5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>46</v>
+      </c>
       <c r="B6">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
       <c r="B7">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
       <c r="B8">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>49</v>
+      </c>
       <c r="B9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>50</v>
+      </c>
       <c r="B10">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>52</v>
+      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>53</v>
+      </c>
       <c r="B13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>54</v>
+      </c>
       <c r="B14">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>131</v>
+      </c>
       <c r="B15">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>132</v>
+      </c>
       <c r="B16">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>133</v>
+      </c>
       <c r="B17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>134</v>
+      </c>
       <c r="B18">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>135</v>
+      </c>
       <c r="B19">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>136</v>
+      </c>
       <c r="B20">
         <v>0</v>
       </c>
@@ -2956,12 +3694,30 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="6" width="30.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>52</v>
+        <v>137</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -2979,7 +3735,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3009,7 +3765,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3017,7 +3773,7 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -3025,7 +3781,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -3033,76 +3789,112 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>40</v>
+      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>41</v>
+      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>45</v>
+      </c>
       <c r="B27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>46</v>
+      </c>
       <c r="B28">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>47</v>
+      </c>
       <c r="B29">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>48</v>
+      </c>
       <c r="B30">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>49</v>
+      </c>
       <c r="B31">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>50</v>
+      </c>
       <c r="B32">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>51</v>
+      </c>
       <c r="B33">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>52</v>
+      </c>
       <c r="B34">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>53</v>
+      </c>
       <c r="B35">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>54</v>
+      </c>
       <c r="B36">
         <v>0</v>
       </c>
@@ -3126,7 +3918,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3156,7 +3948,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3164,33 +3956,48 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
       <c r="B9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
       <c r="B10">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>60</v>
+      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>61</v>
+      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>62</v>
+      </c>
       <c r="B13">
         <v>0</v>
       </c>
@@ -3214,7 +4021,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3244,7 +4051,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3252,38 +4059,56 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>65</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>66</v>
+      </c>
       <c r="B10">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>67</v>
+      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>68</v>
+      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>69</v>
+      </c>
       <c r="B13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>70</v>
+      </c>
       <c r="B14">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>71</v>
+      </c>
       <c r="B15">
         <v>0</v>
       </c>
@@ -3307,7 +4132,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3337,7 +4162,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3345,38 +4170,56 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>75</v>
+      </c>
       <c r="B9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>76</v>
+      </c>
       <c r="B10">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>77</v>
+      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>78</v>
+      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>79</v>
+      </c>
       <c r="B13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>80</v>
+      </c>
       <c r="B14">
         <v>0</v>
       </c>
@@ -3400,7 +4243,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3430,7 +4273,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3438,18 +4281,24 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>84</v>
+      </c>
       <c r="B9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>85</v>
+      </c>
       <c r="B10">
         <v>0</v>
       </c>
@@ -3473,7 +4322,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3503,7 +4352,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3511,91 +4360,136 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>31</v>
+        <v>88</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>89</v>
+      </c>
       <c r="B9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>90</v>
+      </c>
       <c r="B10">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>91</v>
+      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>92</v>
+      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>93</v>
+      </c>
       <c r="B13">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>45</v>
+      </c>
       <c r="B27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>46</v>
+      </c>
       <c r="B28">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>47</v>
+      </c>
       <c r="B29">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>48</v>
+      </c>
       <c r="B30">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>49</v>
+      </c>
       <c r="B31">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>50</v>
+      </c>
       <c r="B32">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>51</v>
+      </c>
       <c r="B33">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>52</v>
+      </c>
       <c r="B34">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>53</v>
+      </c>
       <c r="B35">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>54</v>
+      </c>
       <c r="B36">
         <v>0</v>
       </c>
@@ -3619,7 +4513,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3649,7 +4543,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
-        <v>33</v>
+        <v>95</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3657,43 +4551,64 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>97</v>
+      </c>
       <c r="B9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>98</v>
+      </c>
       <c r="B10">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>99</v>
+      </c>
       <c r="B11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>100</v>
+      </c>
       <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>101</v>
+      </c>
       <c r="B13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>102</v>
+      </c>
       <c r="B14">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>103</v>
+      </c>
       <c r="B15">
         <v>0</v>
       </c>
@@ -3717,34 +4632,34 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="2" t="s">
-        <v>35</v>
+        <v>104</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>37</v>
+        <v>106</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>38</v>
+        <v>107</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>39</v>
+        <v>108</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>40</v>
+        <v>109</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>41</v>
+        <v>110</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>42</v>
+        <v>111</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>43</v>
+        <v>112</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>44</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>